<commit_message>
Element and label pairs histograms, excel, done
</commit_message>
<xml_diff>
--- a/20240304_ternary_test copy/output/20240304_ternary_test copy_label_pairs.xlsx
+++ b/20240304_ternary_test copy/output/20240304_ternary_test copy_label_pairs.xlsx
@@ -8,15 +8,15 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ir1-Ge1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge1-Ge1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eu1-Ge1" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ni1-Ni1B" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ce1-Ni1B" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge1A-Ge1A" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ni1-Ge1A" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ni1B-Ni1B" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ni1B-Ge1A" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ce1-Ge1A" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eu1-Ge1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge1-Ge1" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ni1-Ge1A" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ni1-Ni1B" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ce1-Ge1A" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ni1B-Ge1A" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge1A-Ge1A" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ni1B-Ni1B" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ce1-Ni1B" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ru1-Ge1" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ce1-Ge1" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
@@ -620,6 +620,52 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Atomic Mixing</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>300171.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3.182</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>full_occupancy</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -675,52 +721,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>File</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Distance</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Atomic Mixing</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>300171.cif</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>3.182</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>full_occupancy</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -800,6 +800,52 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>2.477</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>full_occupancy_atomic_mixing</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Atomic Mixing</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1040392.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>3.141</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -813,7 +859,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -859,7 +905,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -892,7 +938,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.477</v>
+        <v>2.226</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -905,7 +951,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -949,50 +995,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>File</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Distance</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Atomic Mixing</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1040392.cif</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>2.226</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>full_occupancy_atomic_mixing</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>